<commit_message>
Rede neural recorrente com estado oculto inicializado
</commit_message>
<xml_diff>
--- a/robot-data/KrigingVsg-/content/KrigingMetrics.xlsx
+++ b/robot-data/KrigingVsg-/content/KrigingMetrics.xlsx
@@ -9,9 +9,6 @@
   <sheets>
     <sheet name="gaussian" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="spherical" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="hole-effect" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="power" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="linear" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,28 +473,28 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.9470832232826287</v>
+        <v>0.9526035159631084</v>
       </c>
       <c r="B2" t="n">
-        <v>0.007305346090802296</v>
+        <v>0.006540467626951996</v>
       </c>
       <c r="C2" t="n">
-        <v>1469389626930.948</v>
+        <v>1074474894504.67</v>
       </c>
       <c r="D2" t="n">
-        <v>0.08547131735735852</v>
+        <v>0.08087315764177874</v>
       </c>
       <c r="E2" t="n">
-        <v>-1.855174868405891</v>
+        <v>-1.768530225380494</v>
       </c>
       <c r="F2" t="n">
-        <v>0.06363152085395406</v>
+        <v>0.06258678623498617</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3915647894911551</v>
+        <v>0.3882036573321304</v>
       </c>
       <c r="H2" t="n">
-        <v>0.25225289067512</v>
+        <v>0.2501735122569657</v>
       </c>
     </row>
   </sheetData>
@@ -558,274 +555,28 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.999896388196305</v>
+        <v>0.9999602836176804</v>
       </c>
       <c r="B2" t="n">
-        <v>1.430397185993739e-05</v>
+        <v>5.480653641289662e-06</v>
       </c>
       <c r="C2" t="n">
-        <v>667038396420.2053</v>
+        <v>445807741304.9562</v>
       </c>
       <c r="D2" t="n">
-        <v>0.003782059208941261</v>
+        <v>0.002341079588841367</v>
       </c>
       <c r="E2" t="n">
-        <v>-11.39820441383729</v>
+        <v>-10.82653452912622</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2763111329678883</v>
+        <v>0.2673565857036573</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8101150834562716</v>
+        <v>0.7980138665907914</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5256530537986898</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>r2_training</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>mse_training</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>mape_training</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>rmse_training</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>r2_test</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>mse_test</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>mape_test</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>rmse_test</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>-19.88618147766194</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2.883410397888737</v>
-      </c>
-      <c r="C2" t="n">
-        <v>648648204417252.5</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1.698060775675811</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-211.7386875294562</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.741175884449894</v>
-      </c>
-      <c r="G2" t="n">
-        <v>3.104409427967257</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2.177424139769258</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>r2_training</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>mse_training</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>mape_training</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>rmse_training</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>r2_test</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>mse_test</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>mape_test</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>rmse_test</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>-14.23519737442661</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2.103272279343732</v>
-      </c>
-      <c r="C2" t="n">
-        <v>707898824813432.9</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1.450266278772189</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-103.2232078965799</v>
-      </c>
-      <c r="F2" t="n">
-        <v>2.322758336143503</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2.337642179132583</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1.524059820395349</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>r2_training</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>mse_training</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>mape_training</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>rmse_training</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>r2_test</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>mse_test</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>mape_test</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>rmse_test</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>0.8885812041466276</v>
-      </c>
-      <c r="B2" t="n">
-        <v>0.0153817544306725</v>
-      </c>
-      <c r="C2" t="n">
-        <v>945948115204.8607</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.1240232011789427</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-15.70885607173083</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.3723799671043168</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.9992641938103836</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.610229438084002</v>
+        <v>0.5170653592184041</v>
       </c>
     </row>
   </sheetData>

</xml_diff>